<commit_message>
Add all compressed videos, remove size exclusions
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/prop/translation/industry-solutions-new.xlsx
+++ b/prop/translation/industry-solutions-new.xlsx
@@ -270,7 +270,7 @@
     <t>University</t>
   </si>
   <si>
-    <t>大学</t>
+    <t>高校</t>
   </si>
   <si>
     <t>university</t>
@@ -295,7 +295,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -313,6 +313,11 @@
     <font>
       <sz val="11"/>
       <name val="Inter"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="宋体"/>
       <charset val="134"/>
     </font>
     <font>
@@ -812,137 +817,137 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -951,6 +956,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1533,7 +1541,7 @@
       <c r="A21" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="4" t="s">
         <v>61</v>
       </c>
       <c r="C21" s="3" t="s">

</xml_diff>